<commit_message>
merging finnhub with main
merging finnhub with main to get updated market data
</commit_message>
<xml_diff>
--- a/data/processed/market/stock_data.xlsx
+++ b/data/processed/market/stock_data.xlsx
@@ -451,111 +451,111 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-02-10T00:00:00.000Z</t>
+          <t>2026-02-26T00:00:00.000Z</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>191.38</v>
+        <v>194.27</v>
       </c>
       <c r="C2" t="n">
-        <v>192.48</v>
+        <v>194.29</v>
       </c>
       <c r="D2" t="n">
-        <v>188.12</v>
+        <v>184.315</v>
       </c>
       <c r="E2" t="n">
-        <v>188.54</v>
+        <v>184.89</v>
       </c>
       <c r="F2" t="n">
-        <v>136764825</v>
+        <v>360807907</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-02-11T00:00:00.000Z</t>
+          <t>2026-02-27T00:00:00.000Z</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>192.45</v>
+        <v>181.25</v>
       </c>
       <c r="C3" t="n">
-        <v>193.26</v>
+        <v>182.59</v>
       </c>
       <c r="D3" t="n">
-        <v>188.77</v>
+        <v>176.38</v>
       </c>
       <c r="E3" t="n">
-        <v>190.05</v>
+        <v>177.19</v>
       </c>
       <c r="F3" t="n">
-        <v>144192685</v>
+        <v>311636494</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-02-12T00:00:00.000Z</t>
+          <t>2026-03-02T00:00:00.000Z</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>193.03</v>
+        <v>175.01</v>
       </c>
       <c r="C4" t="n">
-        <v>193.61</v>
+        <v>183.46</v>
       </c>
       <c r="D4" t="n">
-        <v>186.51</v>
+        <v>174.64</v>
       </c>
       <c r="E4" t="n">
-        <v>186.94</v>
+        <v>182.48</v>
       </c>
       <c r="F4" t="n">
-        <v>189932491</v>
+        <v>209095331</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-02-13T00:00:00.000Z</t>
+          <t>2026-03-03T00:00:00.000Z</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>187.475</v>
+        <v>178.49</v>
       </c>
       <c r="C5" t="n">
-        <v>187.5</v>
+        <v>180.9</v>
       </c>
       <c r="D5" t="n">
-        <v>181.59</v>
+        <v>176.92</v>
       </c>
       <c r="E5" t="n">
-        <v>182.81</v>
+        <v>180.05</v>
       </c>
       <c r="F5" t="n">
-        <v>161888021</v>
+        <v>178099430</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-02-17T00:00:00.000Z</t>
+          <t>2026-03-04T00:00:00.000Z</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>181.75</v>
+        <v>180.44</v>
       </c>
       <c r="C6" t="n">
-        <v>187.15</v>
+        <v>184.7</v>
       </c>
       <c r="D6" t="n">
-        <v>179.18</v>
+        <v>180.06</v>
       </c>
       <c r="E6" t="n">
-        <v>184.97</v>
+        <v>183.04</v>
       </c>
       <c r="F6" t="n">
-        <v>162276860</v>
+        <v>177731198</v>
       </c>
     </row>
   </sheetData>

</xml_diff>